<commit_message>
worked through line 10
</commit_message>
<xml_diff>
--- a/tom_review_2026-09-28/tom_review/state_law_review_workbook.xlsx
+++ b/tom_review_2026-09-28/tom_review/state_law_review_workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Working_Projects\HigherEdLabor\tom_review_2026-09-28\tom_review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{570DB09E-CC2B-4225-9F4C-8ABF98227E7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F70518-E7F6-4C0C-B8CA-11F930800692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="1185" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start here" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6316" uniqueCount="1916">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7599" uniqueCount="1925">
   <si>
     <t>Start here</t>
   </si>
@@ -5832,6 +5832,33 @@
   </si>
   <si>
     <t>Seems like pretty much zero info on donors identity, donation size or how it can be used is given.</t>
+  </si>
+  <si>
+    <t>Neither</t>
+  </si>
+  <si>
+    <t>Not sure about this one, but it seems like the sections regarding reporting and audits went into effect in 2013. Here is the history:  P.A. 13-275 added provision re obligations of executive authority of each state agency for which a foundation is established for principal purpose of coordinated emergency recovery, made a technical change in Subdiv. (3), amended Subdiv. (8) to make full audit requirement applicable to foundation established for principal purpose of coordinated emergency recovery that operated in response to an eligible incident during the fiscal year or with funds that exceeded $100,000 in the aggregate, to exempt such foundation from requirement of full audit for third fiscal year in three-year period for foundations having receipts and earnings of less than $100,000 in each fiscal year if such foundation had completed on its behalf such an audit for any year in any such three-year period, and to require foundation to provide copy of audit report to the Attorney General, and added Subdiv. (10) re which department is deemed the state agency and which official is deemed the executive authority for purposes of section when foundation is established for principal purpose of coordinated emergency recovery, effective July 11, 2013; P.A</t>
+  </si>
+  <si>
+    <t>Sources seem to be conflicting here, but rcfp.org says the actual ruling occurred on the date I provided, slightly before what Claude said, which is when the report is from. "Because the foundation shared management staff, equipment and other resources with the university, it must comply with Georgia’s Sunshine Laws, he said Nov. 14."</t>
+  </si>
+  <si>
+    <t>donors exempt from public discplosure after 2005</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>This has nothing to do with higher ed foundations, it’s a decision regarding a private nonprofit TV broadcaster</t>
+  </si>
+  <si>
+    <t>Partly</t>
+  </si>
+  <si>
+    <t>Seems like claim is supported, though the footnote says this is not a ruling about what counts as confidentials</t>
+  </si>
+  <si>
+    <t>foundations are contracted to perform a governmental function, if a document relates to a gov function then it is subject to foia</t>
   </si>
 </sst>
 </file>
@@ -5850,11 +5877,13 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -6241,629 +6270,629 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A134"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:1" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:1" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="2"/>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="2"/>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="64" spans="1:1" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" s="2"/>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="2"/>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="2"/>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="2"/>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="2"/>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" s="2"/>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" s="2"/>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="2"/>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" s="2"/>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" s="2"/>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>109</v>
       </c>
@@ -6876,7 +6905,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AB94"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
@@ -6892,7 +6921,7 @@
     <col min="28" max="28" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>110</v>
       </c>
@@ -6978,7 +7007,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -7044,7 +7073,7 @@
         <v>1910</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -7110,7 +7139,7 @@
         <v>1911</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -7196,7 +7225,7 @@
         <v>1913</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -7262,7 +7291,7 @@
         <v>1915</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -7324,15 +7353,29 @@
       <c r="U6" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="V6" s="6"/>
-      <c r="W6" s="6"/>
-      <c r="X6" s="6"/>
-      <c r="Y6" s="6"/>
-      <c r="Z6" s="6"/>
-      <c r="AA6" s="6"/>
-      <c r="AB6" s="6"/>
-    </row>
-    <row r="7" spans="1:28" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="V6" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="W6" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="X6" s="8">
+        <v>41436</v>
+      </c>
+      <c r="Y6" s="6" t="s">
+        <v>1916</v>
+      </c>
+      <c r="Z6" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="AA6" s="6">
+        <v>20</v>
+      </c>
+      <c r="AB6" s="6" t="s">
+        <v>1917</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" ht="120" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -7394,15 +7437,29 @@
       <c r="U7" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="V7" s="6"/>
-      <c r="W7" s="6"/>
-      <c r="X7" s="6"/>
-      <c r="Y7" s="6"/>
-      <c r="Z7" s="6"/>
-      <c r="AA7" s="6"/>
-      <c r="AB7" s="6"/>
-    </row>
-    <row r="8" spans="1:28" ht="156.75" x14ac:dyDescent="0.45">
+      <c r="V7" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="W7" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="X7" s="8">
+        <v>37939</v>
+      </c>
+      <c r="Y7" s="6" t="s">
+        <v>1909</v>
+      </c>
+      <c r="Z7" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="AA7" s="6">
+        <v>5</v>
+      </c>
+      <c r="AB7" s="6" t="s">
+        <v>1918</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" ht="195" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -7464,15 +7521,29 @@
       <c r="U8" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="V8" s="6"/>
-      <c r="W8" s="6"/>
-      <c r="X8" s="6"/>
-      <c r="Y8" s="6"/>
-      <c r="Z8" s="6"/>
-      <c r="AA8" s="6"/>
-      <c r="AB8" s="6"/>
-    </row>
-    <row r="9" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+      <c r="V8" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="W8" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="X8" s="6">
+        <v>2005</v>
+      </c>
+      <c r="Y8" s="6" t="s">
+        <v>1909</v>
+      </c>
+      <c r="Z8" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="AA8" s="6">
+        <v>25</v>
+      </c>
+      <c r="AB8" s="6" t="s">
+        <v>1919</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -7516,15 +7587,27 @@
       </c>
       <c r="T9" s="2"/>
       <c r="U9" s="2"/>
-      <c r="V9" s="6"/>
-      <c r="W9" s="6"/>
+      <c r="V9" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="W9" s="6" t="s">
+        <v>1908</v>
+      </c>
       <c r="X9" s="6"/>
-      <c r="Y9" s="6"/>
-      <c r="Z9" s="6"/>
-      <c r="AA9" s="6"/>
-      <c r="AB9" s="6"/>
-    </row>
-    <row r="10" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+      <c r="Y9" s="6" t="s">
+        <v>1916</v>
+      </c>
+      <c r="Z9" s="6" t="s">
+        <v>1920</v>
+      </c>
+      <c r="AA9" s="6">
+        <v>5</v>
+      </c>
+      <c r="AB9" s="6" t="s">
+        <v>1921</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -7584,15 +7667,29 @@
         <v>247</v>
       </c>
       <c r="U10" s="2"/>
-      <c r="V10" s="6"/>
-      <c r="W10" s="6"/>
-      <c r="X10" s="6"/>
-      <c r="Y10" s="6"/>
-      <c r="Z10" s="6"/>
-      <c r="AA10" s="6"/>
-      <c r="AB10" s="6"/>
-    </row>
-    <row r="11" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="V10" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="W10" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="X10" s="8">
+        <v>38387</v>
+      </c>
+      <c r="Y10" s="6" t="s">
+        <v>1914</v>
+      </c>
+      <c r="Z10" s="6" t="s">
+        <v>1922</v>
+      </c>
+      <c r="AA10" s="6">
+        <v>11</v>
+      </c>
+      <c r="AB10" s="6" t="s">
+        <v>1923</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -7638,15 +7735,29 @@
         <v>256</v>
       </c>
       <c r="U11" s="2"/>
-      <c r="V11" s="6"/>
-      <c r="W11" s="6"/>
-      <c r="X11" s="6"/>
-      <c r="Y11" s="6"/>
-      <c r="Z11" s="6"/>
-      <c r="AA11" s="6"/>
-      <c r="AB11" s="6"/>
-    </row>
-    <row r="12" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="V11" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="W11" s="6" t="s">
+        <v>1908</v>
+      </c>
+      <c r="X11" s="8">
+        <v>42864</v>
+      </c>
+      <c r="Y11" s="6" t="s">
+        <v>1914</v>
+      </c>
+      <c r="Z11" s="6" t="s">
+        <v>1922</v>
+      </c>
+      <c r="AA11" s="6">
+        <v>4</v>
+      </c>
+      <c r="AB11" s="6" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -7700,7 +7811,7 @@
       <c r="AA12" s="6"/>
       <c r="AB12" s="6"/>
     </row>
-    <row r="13" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -7770,7 +7881,7 @@
       <c r="AA13" s="6"/>
       <c r="AB13" s="6"/>
     </row>
-    <row r="14" spans="1:28" ht="299.25" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:28" ht="360" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -7840,7 +7951,7 @@
       <c r="AA14" s="6"/>
       <c r="AB14" s="6"/>
     </row>
-    <row r="15" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -7894,7 +8005,7 @@
       <c r="AA15" s="6"/>
       <c r="AB15" s="6"/>
     </row>
-    <row r="16" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -7962,7 +8073,7 @@
       <c r="AA16" s="6"/>
       <c r="AB16" s="6"/>
     </row>
-    <row r="17" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -8016,7 +8127,7 @@
       <c r="AA17" s="6"/>
       <c r="AB17" s="6"/>
     </row>
-    <row r="18" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -8086,7 +8197,7 @@
       <c r="AA18" s="6"/>
       <c r="AB18" s="6"/>
     </row>
-    <row r="19" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -8140,7 +8251,7 @@
       <c r="AA19" s="6"/>
       <c r="AB19" s="6"/>
     </row>
-    <row r="20" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -8194,7 +8305,7 @@
       <c r="AA20" s="6"/>
       <c r="AB20" s="6"/>
     </row>
-    <row r="21" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -8248,7 +8359,7 @@
       <c r="AA21" s="6"/>
       <c r="AB21" s="6"/>
     </row>
-    <row r="22" spans="1:28" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:28" ht="120" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -8318,7 +8429,7 @@
       <c r="AA22" s="6"/>
       <c r="AB22" s="6"/>
     </row>
-    <row r="23" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -8386,7 +8497,7 @@
       <c r="AA23" s="6"/>
       <c r="AB23" s="6"/>
     </row>
-    <row r="24" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -8456,7 +8567,7 @@
       <c r="AA24" s="6"/>
       <c r="AB24" s="6"/>
     </row>
-    <row r="25" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -8510,7 +8621,7 @@
       <c r="AA25" s="6"/>
       <c r="AB25" s="6"/>
     </row>
-    <row r="26" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -8564,7 +8675,7 @@
       <c r="AA26" s="6"/>
       <c r="AB26" s="6"/>
     </row>
-    <row r="27" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -8618,7 +8729,7 @@
       <c r="AA27" s="6"/>
       <c r="AB27" s="6"/>
     </row>
-    <row r="28" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -8670,7 +8781,7 @@
       <c r="AA28" s="6"/>
       <c r="AB28" s="6"/>
     </row>
-    <row r="29" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -8724,7 +8835,7 @@
       <c r="AA29" s="6"/>
       <c r="AB29" s="6"/>
     </row>
-    <row r="30" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -8776,7 +8887,7 @@
       <c r="AA30" s="6"/>
       <c r="AB30" s="6"/>
     </row>
-    <row r="31" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -8830,7 +8941,7 @@
       <c r="AA31" s="6"/>
       <c r="AB31" s="6"/>
     </row>
-    <row r="32" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -8884,7 +8995,7 @@
       <c r="AA32" s="6"/>
       <c r="AB32" s="6"/>
     </row>
-    <row r="33" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -8938,7 +9049,7 @@
       <c r="AA33" s="6"/>
       <c r="AB33" s="6"/>
     </row>
-    <row r="34" spans="1:28" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -8992,7 +9103,7 @@
       <c r="AA34" s="6"/>
       <c r="AB34" s="6"/>
     </row>
-    <row r="35" spans="1:28" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:28" ht="120" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -9060,7 +9171,7 @@
       <c r="AA35" s="6"/>
       <c r="AB35" s="6"/>
     </row>
-    <row r="36" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -9114,7 +9225,7 @@
       <c r="AA36" s="6"/>
       <c r="AB36" s="6"/>
     </row>
-    <row r="37" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -9184,7 +9295,7 @@
       <c r="AA37" s="6"/>
       <c r="AB37" s="6"/>
     </row>
-    <row r="38" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -9254,7 +9365,7 @@
       <c r="AA38" s="6"/>
       <c r="AB38" s="6"/>
     </row>
-    <row r="39" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -9322,7 +9433,7 @@
       <c r="AA39" s="6"/>
       <c r="AB39" s="6"/>
     </row>
-    <row r="40" spans="1:28" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -9376,7 +9487,7 @@
       <c r="AA40" s="6"/>
       <c r="AB40" s="6"/>
     </row>
-    <row r="41" spans="1:28" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:28" ht="180" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -9446,7 +9557,7 @@
       <c r="AA41" s="6"/>
       <c r="AB41" s="6"/>
     </row>
-    <row r="42" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -9516,7 +9627,7 @@
       <c r="AA42" s="6"/>
       <c r="AB42" s="6"/>
     </row>
-    <row r="43" spans="1:28" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -9570,7 +9681,7 @@
       <c r="AA43" s="6"/>
       <c r="AB43" s="6"/>
     </row>
-    <row r="44" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -9636,7 +9747,7 @@
       <c r="AA44" s="6"/>
       <c r="AB44" s="6"/>
     </row>
-    <row r="45" spans="1:28" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:28" ht="120" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -9686,7 +9797,7 @@
       <c r="AA45" s="6"/>
       <c r="AB45" s="6"/>
     </row>
-    <row r="46" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -9734,7 +9845,7 @@
       <c r="AA46" s="6"/>
       <c r="AB46" s="6"/>
     </row>
-    <row r="47" spans="1:28" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:28" ht="135" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -9800,7 +9911,7 @@
       <c r="AA47" s="6"/>
       <c r="AB47" s="6"/>
     </row>
-    <row r="48" spans="1:28" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:28" ht="120" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -9866,7 +9977,7 @@
       <c r="AA48" s="6"/>
       <c r="AB48" s="6"/>
     </row>
-    <row r="49" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -9932,7 +10043,7 @@
       <c r="AA49" s="6"/>
       <c r="AB49" s="6"/>
     </row>
-    <row r="50" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -9982,7 +10093,7 @@
       <c r="AA50" s="6"/>
       <c r="AB50" s="6"/>
     </row>
-    <row r="51" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -10030,7 +10141,7 @@
       <c r="AA51" s="6"/>
       <c r="AB51" s="6"/>
     </row>
-    <row r="52" spans="1:28" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -10096,7 +10207,7 @@
       <c r="AA52" s="6"/>
       <c r="AB52" s="6"/>
     </row>
-    <row r="53" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -10144,7 +10255,7 @@
       <c r="AA53" s="6"/>
       <c r="AB53" s="6"/>
     </row>
-    <row r="54" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -10212,7 +10323,7 @@
       <c r="AA54" s="6"/>
       <c r="AB54" s="6"/>
     </row>
-    <row r="55" spans="1:28" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -10280,7 +10391,7 @@
       <c r="AA55" s="6"/>
       <c r="AB55" s="6"/>
     </row>
-    <row r="56" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -10330,7 +10441,7 @@
       <c r="AA56" s="6"/>
       <c r="AB56" s="6"/>
     </row>
-    <row r="57" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -10398,7 +10509,7 @@
       <c r="AA57" s="6"/>
       <c r="AB57" s="6"/>
     </row>
-    <row r="58" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -10464,7 +10575,7 @@
       <c r="AA58" s="6"/>
       <c r="AB58" s="6"/>
     </row>
-    <row r="59" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -10532,7 +10643,7 @@
       <c r="AA59" s="6"/>
       <c r="AB59" s="6"/>
     </row>
-    <row r="60" spans="1:28" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:28" ht="165" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -10600,7 +10711,7 @@
       <c r="AA60" s="6"/>
       <c r="AB60" s="6"/>
     </row>
-    <row r="61" spans="1:28" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:28" ht="165" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -10668,7 +10779,7 @@
       <c r="AA61" s="6"/>
       <c r="AB61" s="6"/>
     </row>
-    <row r="62" spans="1:28" ht="114" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -10736,7 +10847,7 @@
       <c r="AA62" s="6"/>
       <c r="AB62" s="6"/>
     </row>
-    <row r="63" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -10804,7 +10915,7 @@
       <c r="AA63" s="6"/>
       <c r="AB63" s="6"/>
     </row>
-    <row r="64" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -10872,7 +10983,7 @@
       <c r="AA64" s="6"/>
       <c r="AB64" s="6"/>
     </row>
-    <row r="65" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -10922,7 +11033,7 @@
       <c r="AA65" s="6"/>
       <c r="AB65" s="6"/>
     </row>
-    <row r="66" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -10988,7 +11099,7 @@
       <c r="AA66" s="6"/>
       <c r="AB66" s="6"/>
     </row>
-    <row r="67" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -11054,7 +11165,7 @@
       <c r="AA67" s="6"/>
       <c r="AB67" s="6"/>
     </row>
-    <row r="68" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -11102,7 +11213,7 @@
       <c r="AA68" s="6"/>
       <c r="AB68" s="6"/>
     </row>
-    <row r="69" spans="1:28" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:28" ht="120" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -11150,7 +11261,7 @@
       <c r="AA69" s="6"/>
       <c r="AB69" s="6"/>
     </row>
-    <row r="70" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -11200,7 +11311,7 @@
       <c r="AA70" s="6"/>
       <c r="AB70" s="6"/>
     </row>
-    <row r="71" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -11266,7 +11377,7 @@
       <c r="AA71" s="6"/>
       <c r="AB71" s="6"/>
     </row>
-    <row r="72" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -11328,7 +11439,7 @@
       <c r="AA72" s="6"/>
       <c r="AB72" s="6"/>
     </row>
-    <row r="73" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -11378,7 +11489,7 @@
       <c r="AA73" s="6"/>
       <c r="AB73" s="6"/>
     </row>
-    <row r="74" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -11442,7 +11553,7 @@
       <c r="AA74" s="6"/>
       <c r="AB74" s="6"/>
     </row>
-    <row r="75" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -11504,7 +11615,7 @@
       <c r="AA75" s="6"/>
       <c r="AB75" s="6"/>
     </row>
-    <row r="76" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -11554,7 +11665,7 @@
       <c r="AA76" s="6"/>
       <c r="AB76" s="6"/>
     </row>
-    <row r="77" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>76</v>
       </c>
@@ -11618,7 +11729,7 @@
       <c r="AA77" s="6"/>
       <c r="AB77" s="6"/>
     </row>
-    <row r="78" spans="1:28" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -11668,7 +11779,7 @@
       <c r="AA78" s="6"/>
       <c r="AB78" s="6"/>
     </row>
-    <row r="79" spans="1:28" ht="114" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:28" ht="120" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -11718,7 +11829,7 @@
       <c r="AA79" s="6"/>
       <c r="AB79" s="6"/>
     </row>
-    <row r="80" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -11768,7 +11879,7 @@
       <c r="AA80" s="6"/>
       <c r="AB80" s="6"/>
     </row>
-    <row r="81" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -11830,7 +11941,7 @@
       <c r="AA81" s="6"/>
       <c r="AB81" s="6"/>
     </row>
-    <row r="82" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -11880,7 +11991,7 @@
       <c r="AA82" s="6"/>
       <c r="AB82" s="6"/>
     </row>
-    <row r="83" spans="1:28" ht="114" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:28" ht="165" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -11942,7 +12053,7 @@
       <c r="AA83" s="6"/>
       <c r="AB83" s="6"/>
     </row>
-    <row r="84" spans="1:28" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -11992,7 +12103,7 @@
       <c r="AA84" s="6"/>
       <c r="AB84" s="6"/>
     </row>
-    <row r="85" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -12058,7 +12169,7 @@
       <c r="AA85" s="6"/>
       <c r="AB85" s="6"/>
     </row>
-    <row r="86" spans="1:28" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:28" ht="165" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -12108,7 +12219,7 @@
       <c r="AA86" s="6"/>
       <c r="AB86" s="6"/>
     </row>
-    <row r="87" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -12170,7 +12281,7 @@
       <c r="AA87" s="6"/>
       <c r="AB87" s="6"/>
     </row>
-    <row r="88" spans="1:28" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -12220,7 +12331,7 @@
       <c r="AA88" s="6"/>
       <c r="AB88" s="6"/>
     </row>
-    <row r="89" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -12282,7 +12393,7 @@
       <c r="AA89" s="6"/>
       <c r="AB89" s="6"/>
     </row>
-    <row r="90" spans="1:28" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -12332,7 +12443,7 @@
       <c r="AA90" s="6"/>
       <c r="AB90" s="6"/>
     </row>
-    <row r="91" spans="1:28" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -12382,7 +12493,7 @@
       <c r="AA91" s="6"/>
       <c r="AB91" s="6"/>
     </row>
-    <row r="92" spans="1:28" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -12432,7 +12543,7 @@
       <c r="AA92" s="6"/>
       <c r="AB92" s="6"/>
     </row>
-    <row r="93" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -12494,7 +12605,7 @@
       <c r="AA93" s="6"/>
       <c r="AB93" s="6"/>
     </row>
-    <row r="94" spans="1:28" ht="57" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -12567,7 +12678,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K52"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="45" customWidth="1"/>
@@ -12576,7 +12687,7 @@
     <col min="11" max="11" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>112</v>
       </c>
@@ -12611,7 +12722,7 @@
         <v>1029</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>825</v>
       </c>
@@ -12642,7 +12753,7 @@
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>819</v>
       </c>
@@ -12673,7 +12784,7 @@
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
     </row>
-    <row r="4" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>837</v>
       </c>
@@ -12704,7 +12815,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>138</v>
       </c>
@@ -12735,7 +12846,7 @@
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
     </row>
-    <row r="6" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>147</v>
       </c>
@@ -12766,7 +12877,7 @@
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>169</v>
       </c>
@@ -12797,7 +12908,7 @@
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>178</v>
       </c>
@@ -12828,7 +12939,7 @@
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>579</v>
       </c>
@@ -12859,7 +12970,7 @@
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
     </row>
-    <row r="10" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>572</v>
       </c>
@@ -12890,7 +13001,7 @@
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>854</v>
       </c>
@@ -12921,7 +13032,7 @@
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
     </row>
-    <row r="12" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>195</v>
       </c>
@@ -12952,7 +13063,7 @@
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>226</v>
       </c>
@@ -12983,7 +13094,7 @@
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>866</v>
       </c>
@@ -13014,7 +13125,7 @@
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>248</v>
       </c>
@@ -13045,7 +13156,7 @@
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
     </row>
-    <row r="16" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>257</v>
       </c>
@@ -13076,7 +13187,7 @@
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>233</v>
       </c>
@@ -13107,7 +13218,7 @@
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>623</v>
       </c>
@@ -13138,7 +13249,7 @@
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>277</v>
       </c>
@@ -13169,7 +13280,7 @@
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>311</v>
       </c>
@@ -13200,7 +13311,7 @@
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>906</v>
       </c>
@@ -13231,7 +13342,7 @@
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
     </row>
-    <row r="22" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>630</v>
       </c>
@@ -13262,7 +13373,7 @@
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>882</v>
       </c>
@@ -13293,7 +13404,7 @@
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>636</v>
       </c>
@@ -13324,7 +13435,7 @@
       <c r="J24" s="6"/>
       <c r="K24" s="6"/>
     </row>
-    <row r="25" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>912</v>
       </c>
@@ -13355,7 +13466,7 @@
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
     </row>
-    <row r="26" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>330</v>
       </c>
@@ -13386,7 +13497,7 @@
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>650</v>
       </c>
@@ -13417,7 +13528,7 @@
       <c r="J27" s="6"/>
       <c r="K27" s="6"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>938</v>
       </c>
@@ -13448,7 +13559,7 @@
       <c r="J28" s="6"/>
       <c r="K28" s="6"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>1105</v>
       </c>
@@ -13479,7 +13590,7 @@
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>702</v>
       </c>
@@ -13510,7 +13621,7 @@
       <c r="J30" s="6"/>
       <c r="K30" s="6"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>1110</v>
       </c>
@@ -13541,7 +13652,7 @@
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
     </row>
-    <row r="32" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>675</v>
       </c>
@@ -13572,7 +13683,7 @@
       <c r="J32" s="6"/>
       <c r="K32" s="6"/>
     </row>
-    <row r="33" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>377</v>
       </c>
@@ -13603,7 +13714,7 @@
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
     </row>
-    <row r="34" spans="1:11" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>391</v>
       </c>
@@ -13634,7 +13745,7 @@
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>
     </row>
-    <row r="35" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>336</v>
       </c>
@@ -13665,7 +13776,7 @@
       <c r="J35" s="6"/>
       <c r="K35" s="6"/>
     </row>
-    <row r="36" spans="1:11" ht="57" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>344</v>
       </c>
@@ -13696,7 +13807,7 @@
       <c r="J36" s="6"/>
       <c r="K36" s="6"/>
     </row>
-    <row r="37" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>404</v>
       </c>
@@ -13727,7 +13838,7 @@
       <c r="J37" s="6"/>
       <c r="K37" s="6"/>
     </row>
-    <row r="38" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>418</v>
       </c>
@@ -13758,7 +13869,7 @@
       <c r="J38" s="6"/>
       <c r="K38" s="6"/>
     </row>
-    <row r="39" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>426</v>
       </c>
@@ -13789,7 +13900,7 @@
       <c r="J39" s="6"/>
       <c r="K39" s="6"/>
     </row>
-    <row r="40" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>433</v>
       </c>
@@ -13820,7 +13931,7 @@
       <c r="J40" s="6"/>
       <c r="K40" s="6"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>976</v>
       </c>
@@ -13851,7 +13962,7 @@
       <c r="J41" s="6"/>
       <c r="K41" s="6"/>
     </row>
-    <row r="42" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>776</v>
       </c>
@@ -13882,7 +13993,7 @@
       <c r="J42" s="6"/>
       <c r="K42" s="6"/>
     </row>
-    <row r="43" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>987</v>
       </c>
@@ -13913,7 +14024,7 @@
       <c r="J43" s="6"/>
       <c r="K43" s="6"/>
     </row>
-    <row r="44" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>441</v>
       </c>
@@ -13944,7 +14055,7 @@
       <c r="J44" s="6"/>
       <c r="K44" s="6"/>
     </row>
-    <row r="45" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>461</v>
       </c>
@@ -13975,7 +14086,7 @@
       <c r="J45" s="6"/>
       <c r="K45" s="6"/>
     </row>
-    <row r="46" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>475</v>
       </c>
@@ -14006,7 +14117,7 @@
       <c r="J46" s="6"/>
       <c r="K46" s="6"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>1014</v>
       </c>
@@ -14037,7 +14148,7 @@
       <c r="J47" s="6"/>
       <c r="K47" s="6"/>
     </row>
-    <row r="48" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>483</v>
       </c>
@@ -14068,7 +14179,7 @@
       <c r="J48" s="6"/>
       <c r="K48" s="6"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>519</v>
       </c>
@@ -14099,7 +14210,7 @@
       <c r="J49" s="6"/>
       <c r="K49" s="6"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>541</v>
       </c>
@@ -14130,7 +14241,7 @@
       <c r="J50" s="6"/>
       <c r="K50" s="6"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>528</v>
       </c>
@@ -14161,7 +14272,7 @@
       <c r="J51" s="6"/>
       <c r="K51" s="6"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>551</v>
       </c>
@@ -14201,12 +14312,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:S58"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="19" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>1171</v>
       </c>
@@ -14265,7 +14376,7 @@
         <v>1188</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="313.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:19" ht="405" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>796</v>
       </c>
@@ -14324,7 +14435,7 @@
         <v>1198</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="384.75" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:19" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>462</v>
       </c>
@@ -14383,7 +14494,7 @@
         <v>1203</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="313.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:19" ht="375" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>196</v>
       </c>
@@ -14442,7 +14553,7 @@
         <v>1207</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:19" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>212</v>
       </c>
@@ -14501,7 +14612,7 @@
         <v>1212</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="313.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:19" ht="405" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>585</v>
       </c>
@@ -14560,7 +14671,7 @@
         <v>1214</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="228" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:19" ht="285" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>234</v>
       </c>
@@ -14619,7 +14730,7 @@
         <v>1217</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="370.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:19" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>598</v>
       </c>
@@ -14678,7 +14789,7 @@
         <v>1219</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="228" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:19" ht="285" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>352</v>
       </c>
@@ -14731,7 +14842,7 @@
         <v>1220</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="327.75" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:19" ht="375" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>666</v>
       </c>
@@ -14790,7 +14901,7 @@
         <v>1222</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:19" ht="240" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>365</v>
       </c>
@@ -14849,7 +14960,7 @@
         <v>1225</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="171" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:19" ht="225" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>148</v>
       </c>
@@ -14908,7 +15019,7 @@
         <v>1226</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="242.25" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:19" ht="300" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>155</v>
       </c>
@@ -14967,7 +15078,7 @@
         <v>1227</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:19" ht="150" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>412</v>
       </c>
@@ -15024,7 +15135,7 @@
       </c>
       <c r="S14" s="2"/>
     </row>
-    <row r="15" spans="1:19" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:19" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>740</v>
       </c>
@@ -15083,7 +15194,7 @@
         <v>1228</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:19" ht="240" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>765</v>
       </c>
@@ -15142,7 +15253,7 @@
         <v>1229</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:19" ht="255" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>611</v>
       </c>
@@ -15201,7 +15312,7 @@
         <v>1231</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="228" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:19" ht="270" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>682</v>
       </c>
@@ -15260,7 +15371,7 @@
         <v>1233</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:19" ht="285" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>378</v>
       </c>
@@ -15319,7 +15430,7 @@
         <v>1235</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="228" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:19" ht="315" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>694</v>
       </c>
@@ -15378,7 +15489,7 @@
         <v>1236</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="256.5" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:19" ht="300" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>826</v>
       </c>
@@ -15437,7 +15548,7 @@
         <v>1237</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="327.75" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:19" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>297</v>
       </c>
@@ -15496,7 +15607,7 @@
         <v>1238</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="256.5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:19" ht="330" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>278</v>
       </c>
@@ -15549,7 +15660,7 @@
         <v>1239</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:19" ht="255" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>637</v>
       </c>
@@ -15608,7 +15719,7 @@
         <v>1240</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="171" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:19" ht="210" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>783</v>
       </c>
@@ -15667,7 +15778,7 @@
         <v>1241</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="171" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:19" ht="210" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>703</v>
       </c>
@@ -15726,7 +15837,7 @@
         <v>1243</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="399" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:19" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>729</v>
       </c>
@@ -15785,7 +15896,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="270.75" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:19" ht="300" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>716</v>
       </c>
@@ -15844,7 +15955,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="270.75" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:19" ht="330" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>651</v>
       </c>
@@ -15897,7 +16008,7 @@
         <v>1247</v>
       </c>
     </row>
-    <row r="30" spans="1:19" ht="270.75" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:19" ht="315" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>913</v>
       </c>
@@ -15950,7 +16061,7 @@
         <v>1248</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:19" ht="195" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>179</v>
       </c>
@@ -16009,7 +16120,7 @@
         <v>1251</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:19" ht="225" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>559</v>
       </c>
@@ -16068,7 +16179,7 @@
         <v>1252</v>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="270.75" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:19" ht="345" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>928</v>
       </c>
@@ -16121,7 +16232,7 @@
         <v>1254</v>
       </c>
     </row>
-    <row r="34" spans="1:19" ht="299.25" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:19" ht="405" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>319</v>
       </c>
@@ -16180,7 +16291,7 @@
         <v>1255</v>
       </c>
     </row>
-    <row r="35" spans="1:19" ht="171" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:19" ht="210" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>484</v>
       </c>
@@ -16239,7 +16350,7 @@
         <v>1256</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:19" ht="225" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>497</v>
       </c>
@@ -16298,7 +16409,7 @@
         <v>1258</v>
       </c>
     </row>
-    <row r="37" spans="1:19" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:19" ht="240" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>509</v>
       </c>
@@ -16357,7 +16468,7 @@
         <v>1260</v>
       </c>
     </row>
-    <row r="38" spans="1:19" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:19" ht="255" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>838</v>
       </c>
@@ -16410,7 +16521,7 @@
         <v>1261</v>
       </c>
     </row>
-    <row r="39" spans="1:19" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:19" ht="240" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>1004</v>
       </c>
@@ -16463,7 +16574,7 @@
         <v>1262</v>
       </c>
     </row>
-    <row r="40" spans="1:19" ht="370.5" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:19" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>808</v>
       </c>
@@ -16516,7 +16627,7 @@
         <v>1263</v>
       </c>
     </row>
-    <row r="41" spans="1:19" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:19" ht="210" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>977</v>
       </c>
@@ -16569,7 +16680,7 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="42" spans="1:19" ht="228" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:19" ht="285" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>265</v>
       </c>
@@ -16628,7 +16739,7 @@
         <v>1265</v>
       </c>
     </row>
-    <row r="43" spans="1:19" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:19" ht="180" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>753</v>
       </c>
@@ -16687,7 +16798,7 @@
         <v>1266</v>
       </c>
     </row>
-    <row r="44" spans="1:19" ht="228" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:19" ht="255" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>427</v>
       </c>
@@ -16746,7 +16857,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="45" spans="1:19" ht="242.25" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:19" ht="315" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>542</v>
       </c>
@@ -16803,7 +16914,7 @@
       </c>
       <c r="S45" s="2"/>
     </row>
-    <row r="46" spans="1:19" ht="171" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:19" ht="195" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>227</v>
       </c>
@@ -16862,7 +16973,7 @@
         <v>1268</v>
       </c>
     </row>
-    <row r="47" spans="1:19" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:19" ht="255" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>139</v>
       </c>
@@ -16921,7 +17032,7 @@
         <v>1269</v>
       </c>
     </row>
-    <row r="48" spans="1:19" ht="171" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:19" ht="210" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>624</v>
       </c>
@@ -16980,7 +17091,7 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="49" spans="1:19" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:19" ht="240" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>580</v>
       </c>
@@ -17033,7 +17144,7 @@
         <v>1272</v>
       </c>
     </row>
-    <row r="50" spans="1:19" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:19" ht="240" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>529</v>
       </c>
@@ -17092,7 +17203,7 @@
         <v>1273</v>
       </c>
     </row>
-    <row r="51" spans="1:19" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:19" ht="285" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>656</v>
       </c>
@@ -17151,7 +17262,7 @@
         <v>1274</v>
       </c>
     </row>
-    <row r="52" spans="1:19" ht="256.5" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:19" ht="300" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>944</v>
       </c>
@@ -17210,7 +17321,7 @@
         <v>1275</v>
       </c>
     </row>
-    <row r="53" spans="1:19" ht="270.75" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:19" ht="315" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>855</v>
       </c>
@@ -17263,7 +17374,7 @@
         <v>1276</v>
       </c>
     </row>
-    <row r="54" spans="1:19" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:19" ht="240" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>867</v>
       </c>
@@ -17316,7 +17427,7 @@
         <v>1277</v>
       </c>
     </row>
-    <row r="55" spans="1:19" ht="242.25" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:19" ht="315" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>883</v>
       </c>
@@ -17369,7 +17480,7 @@
         <v>1278</v>
       </c>
     </row>
-    <row r="56" spans="1:19" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:19" ht="300" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>960</v>
       </c>
@@ -17422,7 +17533,7 @@
         <v>1279</v>
       </c>
     </row>
-    <row r="57" spans="1:19" ht="256.5" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:19" ht="345" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>631</v>
       </c>
@@ -17471,7 +17582,7 @@
         <v>1282</v>
       </c>
     </row>
-    <row r="58" spans="1:19" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:19" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>814</v>
       </c>
@@ -17529,12 +17640,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AZ83"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="52" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:52" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>1171</v>
       </c>
@@ -17692,7 +17803,7 @@
         <v>1334</v>
       </c>
     </row>
-    <row r="2" spans="1:52" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:52" ht="165" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>820</v>
       </c>
@@ -17836,7 +17947,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="3" spans="1:52" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:52" ht="225" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>827</v>
       </c>
@@ -17982,7 +18093,7 @@
         <v>1373</v>
       </c>
     </row>
-    <row r="4" spans="1:52" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:52" ht="165" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>839</v>
       </c>
@@ -18124,7 +18235,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="5" spans="1:52" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:52" ht="150" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>849</v>
       </c>
@@ -18268,7 +18379,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="6" spans="1:52" ht="313.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:52" ht="375" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>156</v>
       </c>
@@ -18420,7 +18531,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="7" spans="1:52" ht="171" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:52" ht="210" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>170</v>
       </c>
@@ -18564,7 +18675,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="8" spans="1:52" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:52" ht="300" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>560</v>
       </c>
@@ -18716,7 +18827,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="9" spans="1:52" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:52" ht="135" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>180</v>
       </c>
@@ -18858,7 +18969,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="10" spans="1:52" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:52" ht="225" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>573</v>
       </c>
@@ -19002,7 +19113,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="11" spans="1:52" ht="256.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:52" ht="285" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>856</v>
       </c>
@@ -19146,7 +19257,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="12" spans="1:52" ht="171" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:52" ht="210" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>197</v>
       </c>
@@ -19290,7 +19401,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="13" spans="1:52" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:52" ht="255" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>213</v>
       </c>
@@ -19438,7 +19549,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="14" spans="1:52" ht="256.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:52" ht="345" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>586</v>
       </c>
@@ -19590,7 +19701,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="15" spans="1:52" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:52" ht="195" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>235</v>
       </c>
@@ -19740,7 +19851,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="16" spans="1:52" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:52" ht="270" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>599</v>
       </c>
@@ -19888,7 +19999,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="17" spans="1:52" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:52" ht="180" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>868</v>
       </c>
@@ -20032,7 +20143,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="18" spans="1:52" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:52" ht="150" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>249</v>
       </c>
@@ -20178,7 +20289,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="19" spans="1:52" ht="242.25" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:52" ht="300" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>612</v>
       </c>
@@ -20328,7 +20439,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="20" spans="1:52" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:52" ht="165" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>258</v>
       </c>
@@ -20470,7 +20581,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="21" spans="1:52" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:52" ht="135" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>266</v>
       </c>
@@ -20614,7 +20725,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="22" spans="1:52" ht="114" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:52" ht="135" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>877</v>
       </c>
@@ -20758,7 +20869,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="23" spans="1:52" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:52" ht="240" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>298</v>
       </c>
@@ -20906,7 +21017,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="24" spans="1:52" ht="228" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:52" ht="270" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>279</v>
       </c>
@@ -21054,7 +21165,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="25" spans="1:52" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:52" ht="165" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>292</v>
       </c>
@@ -21196,7 +21307,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="26" spans="1:52" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:52" ht="180" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>312</v>
       </c>
@@ -21344,7 +21455,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="27" spans="1:52" ht="171" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:52" ht="240" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>320</v>
       </c>
@@ -21488,7 +21599,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="28" spans="1:52" ht="171" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:52" ht="255" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>884</v>
       </c>
@@ -21632,7 +21743,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="29" spans="1:52" ht="114" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:52" ht="120" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>895</v>
       </c>
@@ -21770,7 +21881,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="30" spans="1:52" ht="228" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:52" ht="285" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>901</v>
       </c>
@@ -21914,7 +22025,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="31" spans="1:52" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:52" ht="150" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>907</v>
       </c>
@@ -22058,7 +22169,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="32" spans="1:52" ht="285" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:52" ht="345" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>638</v>
       </c>
@@ -22206,7 +22317,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="33" spans="1:52" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:52" ht="225" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>914</v>
       </c>
@@ -22346,7 +22457,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="34" spans="1:52" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:52" ht="135" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>923</v>
       </c>
@@ -22490,7 +22601,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="35" spans="1:52" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:52" ht="135" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>331</v>
       </c>
@@ -22634,7 +22745,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="36" spans="1:52" ht="256.5" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:52" ht="315" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>929</v>
       </c>
@@ -22776,7 +22887,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="37" spans="1:52" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:52" ht="165" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>939</v>
       </c>
@@ -22920,7 +23031,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="38" spans="1:52" ht="114" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:52" ht="150" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>337</v>
       </c>
@@ -23064,7 +23175,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="39" spans="1:52" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:52" ht="135" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>657</v>
       </c>
@@ -23206,7 +23317,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="40" spans="1:52" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:52" ht="210" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>945</v>
       </c>
@@ -23348,7 +23459,7 @@
         <v>1650</v>
       </c>
     </row>
-    <row r="41" spans="1:52" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:52" ht="180" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>667</v>
       </c>
@@ -23494,7 +23605,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="42" spans="1:52" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:52" ht="180" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>345</v>
       </c>
@@ -23640,7 +23751,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="43" spans="1:52" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:52" ht="180" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>366</v>
       </c>
@@ -23786,7 +23897,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="44" spans="1:52" ht="171" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:52" ht="240" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>353</v>
       </c>
@@ -23934,7 +24045,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="45" spans="1:52" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:52" ht="270" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>683</v>
       </c>
@@ -24082,7 +24193,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="46" spans="1:52" ht="171" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:52" ht="210" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>676</v>
       </c>
@@ -24222,7 +24333,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="47" spans="1:52" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:52" ht="240" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>379</v>
       </c>
@@ -24368,7 +24479,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="48" spans="1:52" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:52" ht="240" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>695</v>
       </c>
@@ -24514,7 +24625,7 @@
         <v>1650</v>
       </c>
     </row>
-    <row r="49" spans="1:52" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:52" ht="255" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>704</v>
       </c>
@@ -24660,7 +24771,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="50" spans="1:52" ht="327.75" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:52" ht="390" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>717</v>
       </c>
@@ -24804,7 +24915,7 @@
         <v>1373</v>
       </c>
     </row>
-    <row r="51" spans="1:52" ht="270.75" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:52" ht="315" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>730</v>
       </c>
@@ -24948,7 +25059,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="52" spans="1:52" ht="114" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:52" ht="135" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>392</v>
       </c>
@@ -25092,7 +25203,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="53" spans="1:52" ht="114" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:52" ht="135" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>400</v>
       </c>
@@ -25236,7 +25347,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="54" spans="1:52" ht="270.75" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:52" ht="315" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>956</v>
       </c>
@@ -25380,7 +25491,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="55" spans="1:52" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:52" ht="165" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>741</v>
       </c>
@@ -25526,7 +25637,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="56" spans="1:52" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:52" ht="180" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>405</v>
       </c>
@@ -25674,7 +25785,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="57" spans="1:52" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:52" ht="165" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>419</v>
       </c>
@@ -25816,7 +25927,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="58" spans="1:52" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:52" ht="165" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>961</v>
       </c>
@@ -25960,7 +26071,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="59" spans="1:52" ht="114" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:52" ht="135" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>754</v>
       </c>
@@ -26100,7 +26211,7 @@
         <v>1373</v>
       </c>
     </row>
-    <row r="60" spans="1:52" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:52" ht="240" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>971</v>
       </c>
@@ -26244,7 +26355,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="61" spans="1:52" ht="171" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:52" ht="195" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>434</v>
       </c>
@@ -26392,7 +26503,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="62" spans="1:52" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:52" ht="240" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>766</v>
       </c>
@@ -26538,7 +26649,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="63" spans="1:52" ht="114" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:52" ht="120" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>978</v>
       </c>
@@ -26678,7 +26789,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="64" spans="1:52" ht="171" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:52" ht="195" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>784</v>
       </c>
@@ -26828,7 +26939,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="65" spans="1:52" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:52" ht="225" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>777</v>
       </c>
@@ -26970,7 +27081,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="66" spans="1:52" ht="114" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:52" ht="135" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>988</v>
       </c>
@@ -27108,7 +27219,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="67" spans="1:52" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:52" ht="105" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>994</v>
       </c>
@@ -27246,7 +27357,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="68" spans="1:52" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:52" ht="180" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>442</v>
       </c>
@@ -27396,7 +27507,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="69" spans="1:52" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:52" ht="135" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>449</v>
       </c>
@@ -27540,7 +27651,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="70" spans="1:52" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:52" ht="210" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>454</v>
       </c>
@@ -27686,7 +27797,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="71" spans="1:52" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:52" ht="165" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>797</v>
       </c>
@@ -27836,7 +27947,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="72" spans="1:52" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:52" ht="240" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>463</v>
       </c>
@@ -27986,7 +28097,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="73" spans="1:52" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:52" ht="270" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>999</v>
       </c>
@@ -28130,7 +28241,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="74" spans="1:52" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:52" ht="240" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>476</v>
       </c>
@@ -28276,7 +28387,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="75" spans="1:52" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:52" ht="240" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>1005</v>
       </c>
@@ -28416,7 +28527,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="76" spans="1:52" ht="114" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:52" ht="150" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>485</v>
       </c>
@@ -28562,7 +28673,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="77" spans="1:52" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:52" ht="180" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>498</v>
       </c>
@@ -28704,7 +28815,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="78" spans="1:52" ht="171" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:52" ht="210" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>510</v>
       </c>
@@ -28850,7 +28961,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="79" spans="1:52" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:52" ht="165" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>1015</v>
       </c>
@@ -28994,7 +29105,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="80" spans="1:52" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:52" ht="105" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>520</v>
       </c>
@@ -29138,7 +29249,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="81" spans="1:52" ht="299.25" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:52" ht="360" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>530</v>
       </c>
@@ -29282,7 +29393,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="82" spans="1:52" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:52" ht="135" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>543</v>
       </c>
@@ -29426,7 +29537,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="83" spans="1:52" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:52" ht="225" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>552</v>
       </c>

</xml_diff>